<commit_message>
Add data-table limit-row validation driven by embedded 限值 rules.
Replace manual column/whole-table range prompts with one 数据校验 button that reads the 限值 row, keep sample-id import from overwriting it, and gate Word output behind a session-only checkbox.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/data_tables/5点法.xlsx
+++ b/templates/data_tables/5点法.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ikaruga/Desktop/Reach/report creator/templates/data_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA5CBAE-68D7-6846-AA6C-F98C7019A70F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA391EC-91CE-1C44-B5A3-EC9712639581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="7">
   <si>
     <t>-40°C</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -43,6 +43,10 @@
   </si>
   <si>
     <t>16V</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>限值</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -400,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="19.59765625" style="1" bestFit="1" customWidth="1"/>
@@ -408,7 +412,7 @@
     <col min="11" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10">
+    <row r="1" spans="1:10">
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
@@ -425,7 +429,7 @@
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
     </row>
-    <row r="2" spans="2:10" ht="15">
+    <row r="2" spans="1:10" ht="15">
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
@@ -452,6 +456,11 @@
       </c>
       <c r="J2" s="2" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>